<commit_message>
feat(sizing): implement 3-Tier Execution Framework (3 Lots 1-OTM, 4 Lots 2-OTM Super-Trend, 2 Lots ATM)
- Add is_super_trend_setup to detect high-velocity trendline & OR-30 expansions
- Add resolve_strike_and_lots to dynamically enforce the 3-Tier Execution Framework
- Tier 1: 3 Lots with 1-OTM for general daily setups
- Tier 2: 4 Lots with 2-OTM for Super-Trend days
- Tier 3: 2 Lots with ATM for expensive/fresh contracts
- Update option_plan, estimated_plan, alert bodies, and Excel logs with tier tags
- Verify 19 backend unit tests passing
</commit_message>
<xml_diff>
--- a/trades/by_strategy/breakout_and_retest.xlsx
+++ b/trades/by_strategy/breakout_and_retest.xlsx
@@ -538,7 +538,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -713,7 +713,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -774,22 +774,22 @@
         <v>195.3</v>
       </c>
       <c r="T2" s="6" t="n">
-        <v>11436</v>
+        <v>22872</v>
       </c>
       <c r="U2" s="6" t="n">
-        <v>12694</v>
+        <v>25389</v>
       </c>
       <c r="V2" s="7" t="n">
-        <v>1188</v>
+        <v>2424</v>
       </c>
       <c r="W2" s="8" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z2" s="3" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -978,22 +978,22 @@
         <v>162.23</v>
       </c>
       <c r="T4" s="6" t="n">
-        <v>11926</v>
+        <v>23851</v>
       </c>
       <c r="U4" s="6" t="n">
-        <v>10545</v>
+        <v>21090</v>
       </c>
       <c r="V4" s="17" t="n">
-        <v>-1448</v>
+        <v>-2849</v>
       </c>
       <c r="W4" s="18" t="n">
-        <v>-12.1</v>
+        <v>-11.9</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22900 PE</t>
+          <t>NIFTY 22850 PE</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
@@ -1074,28 +1074,28 @@
         </is>
       </c>
       <c r="R5" s="11" t="n">
-        <v>195.25</v>
+        <v>170.75</v>
       </c>
       <c r="S5" s="11" t="n">
-        <v>194.88</v>
+        <v>170.38</v>
       </c>
       <c r="T5" s="13" t="n">
-        <v>12691</v>
+        <v>33296</v>
       </c>
       <c r="U5" s="13" t="n">
-        <v>12667</v>
+        <v>33224</v>
       </c>
       <c r="V5" s="20" t="n">
-        <v>-95</v>
+        <v>-181</v>
       </c>
       <c r="W5" s="21" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
       <c r="X5" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y5" s="9" t="n">
-        <v>65</v>
+        <v>195</v>
       </c>
       <c r="Z5" s="10" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22950 PE</t>
+          <t>NIFTY 22900 PE</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1176,28 +1176,28 @@
         </is>
       </c>
       <c r="R6" s="4" t="n">
-        <v>194.4</v>
+        <v>170.04</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>193.99</v>
+        <v>169.63</v>
       </c>
       <c r="T6" s="6" t="n">
-        <v>25272</v>
+        <v>33158</v>
       </c>
       <c r="U6" s="6" t="n">
-        <v>25219</v>
+        <v>33078</v>
       </c>
       <c r="V6" s="17" t="n">
-        <v>-147</v>
+        <v>-189</v>
       </c>
       <c r="W6" s="18" t="n">
         <v>-0.6</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z6" s="3" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>PDH Support Flip</t>
+          <t>PDH Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23100 CE</t>
+          <t>NIFTY 23200 CE</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
@@ -1278,22 +1278,22 @@
         </is>
       </c>
       <c r="R7" s="11" t="n">
-        <v>115.13</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="S7" s="11" t="n">
-        <v>131.37</v>
+        <v>85.19</v>
       </c>
       <c r="T7" s="13" t="n">
-        <v>14967</v>
+        <v>9536</v>
       </c>
       <c r="U7" s="13" t="n">
-        <v>17078</v>
+        <v>11075</v>
       </c>
       <c r="V7" s="14" t="n">
-        <v>2033</v>
+        <v>1472</v>
       </c>
       <c r="W7" s="15" t="n">
-        <v>13.6</v>
+        <v>15.4</v>
       </c>
       <c r="X7" s="9" t="n">
         <v>2</v>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23100 CE</t>
+          <t>NIFTY 23200 CE</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1380,22 +1380,22 @@
         </is>
       </c>
       <c r="R8" s="4" t="n">
-        <v>125.68</v>
+        <v>81.22</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>107.23</v>
+        <v>67.58</v>
       </c>
       <c r="T8" s="6" t="n">
-        <v>16338</v>
+        <v>10559</v>
       </c>
       <c r="U8" s="6" t="n">
-        <v>13940</v>
+        <v>8785</v>
       </c>
       <c r="V8" s="17" t="n">
-        <v>-2473</v>
+        <v>-1838</v>
       </c>
       <c r="W8" s="18" t="n">
-        <v>-15.1</v>
+        <v>-17.4</v>
       </c>
       <c r="X8" s="2" t="n">
         <v>2</v>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>PDH Support Flip</t>
+          <t>PDH Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22800 CE</t>
+          <t>NIFTY 22900 CE</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
@@ -1482,28 +1482,28 @@
         </is>
       </c>
       <c r="R9" s="11" t="n">
-        <v>137.01</v>
+        <v>94.22</v>
       </c>
       <c r="S9" s="11" t="n">
-        <v>217.9</v>
+        <v>159.33</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>8906</v>
+        <v>12249</v>
       </c>
       <c r="U9" s="13" t="n">
-        <v>14164</v>
+        <v>20713</v>
       </c>
       <c r="V9" s="14" t="n">
-        <v>5187</v>
+        <v>8382</v>
       </c>
       <c r="W9" s="15" t="n">
-        <v>58.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="X9" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y9" s="9" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z9" s="10" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22500 PE</t>
+          <t>NIFTY 22400 PE</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1584,28 +1584,28 @@
         </is>
       </c>
       <c r="R10" s="4" t="n">
-        <v>71.77</v>
+        <v>33.27</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>83.88</v>
+        <v>40.3</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>9330</v>
+        <v>6488</v>
       </c>
       <c r="U10" s="6" t="n">
-        <v>10904</v>
+        <v>7858</v>
       </c>
       <c r="V10" s="7" t="n">
-        <v>1508</v>
+        <v>1310</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>16.2</v>
+        <v>20.2</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z10" s="3" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22500 CE</t>
+          <t>NIFTY 22600 CE</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="R11" s="11" t="n">
-        <v>138.73</v>
+        <v>96.29000000000001</v>
       </c>
       <c r="S11" s="11" t="n">
-        <v>171.78</v>
+        <v>121.92</v>
       </c>
       <c r="T11" s="13" t="n">
-        <v>9017</v>
+        <v>12518</v>
       </c>
       <c r="U11" s="13" t="n">
-        <v>11166</v>
+        <v>15850</v>
       </c>
       <c r="V11" s="14" t="n">
-        <v>2081</v>
+        <v>3257</v>
       </c>
       <c r="W11" s="15" t="n">
-        <v>23.1</v>
+        <v>26</v>
       </c>
       <c r="X11" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y11" s="9" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z11" s="10" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22450 PE</t>
+          <t>NIFTY 22350 PE</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1788,28 +1788,28 @@
         </is>
       </c>
       <c r="R12" s="4" t="n">
-        <v>145.25</v>
+        <v>100.98</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>222.17</v>
+        <v>163.09</v>
       </c>
       <c r="T12" s="6" t="n">
-        <v>9441</v>
+        <v>13127</v>
       </c>
       <c r="U12" s="6" t="n">
-        <v>14441</v>
+        <v>21202</v>
       </c>
       <c r="V12" s="7" t="n">
-        <v>4928</v>
+        <v>7991</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>52.2</v>
+        <v>60.9</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z12" s="3" t="inlineStr">
         <is>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22500 PE</t>
+          <t>NIFTY 22400 PE</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
@@ -1890,28 +1890,28 @@
         </is>
       </c>
       <c r="R13" s="11" t="n">
-        <v>147.5</v>
+        <v>102.9</v>
       </c>
       <c r="S13" s="11" t="n">
-        <v>170.81</v>
+        <v>121.28</v>
       </c>
       <c r="T13" s="13" t="n">
-        <v>9588</v>
+        <v>13377</v>
       </c>
       <c r="U13" s="13" t="n">
-        <v>11103</v>
+        <v>15766</v>
       </c>
       <c r="V13" s="14" t="n">
-        <v>1448</v>
+        <v>2314</v>
       </c>
       <c r="W13" s="15" t="n">
-        <v>15.1</v>
+        <v>17.3</v>
       </c>
       <c r="X13" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y13" s="9" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z13" s="10" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22550 PE</t>
+          <t>NIFTY 22500 PE</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -1992,28 +1992,28 @@
         </is>
       </c>
       <c r="R14" s="4" t="n">
-        <v>153.06</v>
+        <v>129.62</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>128.78</v>
+        <v>107.95</v>
       </c>
       <c r="T14" s="6" t="n">
-        <v>9949</v>
+        <v>16851</v>
       </c>
       <c r="U14" s="6" t="n">
-        <v>8371</v>
+        <v>14034</v>
       </c>
       <c r="V14" s="17" t="n">
-        <v>-1642</v>
+        <v>-2892</v>
       </c>
       <c r="W14" s="18" t="n">
-        <v>-16.5</v>
+        <v>-17.2</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z14" s="3" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22650 CE</t>
+          <t>NIFTY 22750 CE</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
@@ -2196,28 +2196,28 @@
         </is>
       </c>
       <c r="R16" s="4" t="n">
-        <v>192.09</v>
+        <v>146.03</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>172.33</v>
+        <v>129.6</v>
       </c>
       <c r="T16" s="6" t="n">
-        <v>24972</v>
+        <v>37968</v>
       </c>
       <c r="U16" s="6" t="n">
-        <v>22403</v>
+        <v>33696</v>
       </c>
       <c r="V16" s="17" t="n">
-        <v>-2659</v>
+        <v>-4384</v>
       </c>
       <c r="W16" s="18" t="n">
-        <v>-10.6</v>
+        <v>-11.5</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z16" s="3" t="inlineStr">
         <is>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>PDH Support Flip</t>
+          <t>PDH Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22650 CE</t>
+          <t>NIFTY 22750 CE</t>
         </is>
       </c>
       <c r="Q17" s="9" t="inlineStr">
@@ -2298,28 +2298,28 @@
         </is>
       </c>
       <c r="R17" s="11" t="n">
-        <v>184.24</v>
+        <v>139.49</v>
       </c>
       <c r="S17" s="11" t="n">
-        <v>202.73</v>
+        <v>154.79</v>
       </c>
       <c r="T17" s="13" t="n">
-        <v>23951</v>
+        <v>36267</v>
       </c>
       <c r="U17" s="13" t="n">
-        <v>26355</v>
+        <v>40245</v>
       </c>
       <c r="V17" s="14" t="n">
-        <v>2309</v>
+        <v>3858</v>
       </c>
       <c r="W17" s="15" t="n">
-        <v>9.6</v>
+        <v>10.6</v>
       </c>
       <c r="X17" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y17" s="9" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z17" s="10" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22500 PE</t>
+          <t>NIFTY 22450 PE</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2400,28 +2400,28 @@
         </is>
       </c>
       <c r="R18" s="4" t="n">
-        <v>150.75</v>
+        <v>126.18</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>236.79</v>
+        <v>204.29</v>
       </c>
       <c r="T18" s="6" t="n">
-        <v>9799</v>
+        <v>16403</v>
       </c>
       <c r="U18" s="6" t="n">
-        <v>15391</v>
+        <v>26558</v>
       </c>
       <c r="V18" s="7" t="n">
-        <v>5519</v>
+        <v>10062</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>56.3</v>
+        <v>61.3</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z18" s="3" t="inlineStr">
         <is>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="P19" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22850 PE</t>
+          <t>NIFTY 22750 PE</t>
         </is>
       </c>
       <c r="Q19" s="9" t="inlineStr">
@@ -2502,28 +2502,28 @@
         </is>
       </c>
       <c r="R19" s="11" t="n">
-        <v>69.90000000000001</v>
+        <v>29.08</v>
       </c>
       <c r="S19" s="11" t="n">
-        <v>88.03</v>
+        <v>37.52</v>
       </c>
       <c r="T19" s="13" t="n">
-        <v>9087</v>
+        <v>5671</v>
       </c>
       <c r="U19" s="13" t="n">
-        <v>11444</v>
+        <v>7316</v>
       </c>
       <c r="V19" s="14" t="n">
-        <v>2289</v>
+        <v>1586</v>
       </c>
       <c r="W19" s="15" t="n">
-        <v>25.2</v>
+        <v>28</v>
       </c>
       <c r="X19" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y19" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z19" s="10" t="inlineStr">
         <is>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23450 CE</t>
+          <t>NIFTY 23500 CE</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -2604,22 +2604,22 @@
         </is>
       </c>
       <c r="R20" s="4" t="n">
-        <v>128.95</v>
+        <v>106.14</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>116.5</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="T20" s="6" t="n">
-        <v>16764</v>
+        <v>13798</v>
       </c>
       <c r="U20" s="6" t="n">
-        <v>15145</v>
+        <v>12359</v>
       </c>
       <c r="V20" s="17" t="n">
-        <v>-1695</v>
+        <v>-1510</v>
       </c>
       <c r="W20" s="18" t="n">
-        <v>-10.1</v>
+        <v>-10.9</v>
       </c>
       <c r="X20" s="2" t="n">
         <v>2</v>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="P21" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23400 PE</t>
+          <t>NIFTY 23300 PE</t>
         </is>
       </c>
       <c r="Q21" s="9" t="inlineStr">
@@ -2706,28 +2706,28 @@
         </is>
       </c>
       <c r="R21" s="11" t="n">
-        <v>155.93</v>
+        <v>109.2</v>
       </c>
       <c r="S21" s="11" t="n">
-        <v>193.44</v>
+        <v>139.1</v>
       </c>
       <c r="T21" s="13" t="n">
-        <v>10135</v>
+        <v>28392</v>
       </c>
       <c r="U21" s="13" t="n">
-        <v>12574</v>
+        <v>36166</v>
       </c>
       <c r="V21" s="14" t="n">
-        <v>2369</v>
+        <v>7663</v>
       </c>
       <c r="W21" s="15" t="n">
-        <v>23.4</v>
+        <v>27</v>
       </c>
       <c r="X21" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y21" s="9" t="n">
-        <v>65</v>
+        <v>260</v>
       </c>
       <c r="Z21" s="10" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>PDH Support Flip</t>
+          <t>PDH Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23400 CE</t>
+          <t>NIFTY 23500 CE</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
@@ -2808,28 +2808,28 @@
         </is>
       </c>
       <c r="R22" s="4" t="n">
-        <v>62.35</v>
+        <v>24.77</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>46.34</v>
+        <v>16.54</v>
       </c>
       <c r="T22" s="6" t="n">
-        <v>8106</v>
+        <v>6440</v>
       </c>
       <c r="U22" s="6" t="n">
-        <v>6024</v>
+        <v>4300</v>
       </c>
       <c r="V22" s="17" t="n">
-        <v>-2141</v>
+        <v>-2196</v>
       </c>
       <c r="W22" s="18" t="n">
-        <v>-26.4</v>
+        <v>-34.1</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z22" s="3" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="P23" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23200 PE</t>
+          <t>NIFTY 23150 PE</t>
         </is>
       </c>
       <c r="Q23" s="9" t="inlineStr">
@@ -2910,28 +2910,28 @@
         </is>
       </c>
       <c r="R23" s="11" t="n">
-        <v>156.61</v>
+        <v>132.84</v>
       </c>
       <c r="S23" s="11" t="n">
-        <v>171.48</v>
+        <v>146.21</v>
       </c>
       <c r="T23" s="13" t="n">
-        <v>20359</v>
+        <v>25904</v>
       </c>
       <c r="U23" s="13" t="n">
-        <v>22292</v>
+        <v>28511</v>
       </c>
       <c r="V23" s="14" t="n">
-        <v>1845</v>
+        <v>2508</v>
       </c>
       <c r="W23" s="15" t="n">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="X23" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y23" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z23" s="10" t="inlineStr">
         <is>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23400 PE</t>
+          <t>NIFTY 23300 PE</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -3012,28 +3012,28 @@
         </is>
       </c>
       <c r="R24" s="4" t="n">
-        <v>164.16</v>
+        <v>118.2</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>181.37</v>
+        <v>132.06</v>
       </c>
       <c r="T24" s="6" t="n">
-        <v>21341</v>
+        <v>30732</v>
       </c>
       <c r="U24" s="6" t="n">
-        <v>23578</v>
+        <v>34336</v>
       </c>
       <c r="V24" s="7" t="n">
-        <v>2147</v>
+        <v>3494</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>10.1</v>
+        <v>11.4</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z24" s="3" t="inlineStr">
         <is>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="P25" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23300 CE</t>
+          <t>NIFTY 23400 CE</t>
         </is>
       </c>
       <c r="Q25" s="9" t="inlineStr">
@@ -3114,28 +3114,28 @@
         </is>
       </c>
       <c r="R25" s="11" t="n">
-        <v>116.52</v>
+        <v>73.81</v>
       </c>
       <c r="S25" s="11" t="n">
-        <v>139.02</v>
+        <v>90.41</v>
       </c>
       <c r="T25" s="13" t="n">
-        <v>15148</v>
+        <v>14393</v>
       </c>
       <c r="U25" s="13" t="n">
-        <v>18073</v>
+        <v>17630</v>
       </c>
       <c r="V25" s="14" t="n">
-        <v>2846</v>
+        <v>3158</v>
       </c>
       <c r="W25" s="15" t="n">
-        <v>18.8</v>
+        <v>21.9</v>
       </c>
       <c r="X25" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y25" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z25" s="10" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23400 PE</t>
+          <t>NIFTY 23300 PE</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
@@ -3216,28 +3216,28 @@
         </is>
       </c>
       <c r="R26" s="4" t="n">
-        <v>127.87</v>
+        <v>84.7</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>105.88</v>
+        <v>68.17</v>
       </c>
       <c r="T26" s="6" t="n">
-        <v>8312</v>
+        <v>11011</v>
       </c>
       <c r="U26" s="6" t="n">
-        <v>6882</v>
+        <v>8862</v>
       </c>
       <c r="V26" s="17" t="n">
-        <v>-1490</v>
+        <v>-2214</v>
       </c>
       <c r="W26" s="18" t="n">
-        <v>-17.9</v>
+        <v>-20.1</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z26" s="3" t="inlineStr">
         <is>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="P27" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23400 PE</t>
+          <t>NIFTY 23300 PE</t>
         </is>
       </c>
       <c r="Q27" s="9" t="inlineStr">
@@ -3318,28 +3318,28 @@
         </is>
       </c>
       <c r="R27" s="11" t="n">
-        <v>124.37</v>
+        <v>82.19</v>
       </c>
       <c r="S27" s="11" t="n">
-        <v>109.25</v>
+        <v>70.87</v>
       </c>
       <c r="T27" s="13" t="n">
-        <v>16168</v>
+        <v>16027</v>
       </c>
       <c r="U27" s="13" t="n">
-        <v>14202</v>
+        <v>13820</v>
       </c>
       <c r="V27" s="20" t="n">
-        <v>-2040</v>
+        <v>-2281</v>
       </c>
       <c r="W27" s="21" t="n">
-        <v>-12.6</v>
+        <v>-14.2</v>
       </c>
       <c r="X27" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y27" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z27" s="10" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23550 CE</t>
+          <t>NIFTY 23650 CE</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
@@ -3420,22 +3420,22 @@
         </is>
       </c>
       <c r="R28" s="4" t="n">
-        <v>130.25</v>
+        <v>87.92</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>111.71</v>
+        <v>73.78</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>16932</v>
+        <v>11430</v>
       </c>
       <c r="U28" s="6" t="n">
-        <v>14522</v>
+        <v>9591</v>
       </c>
       <c r="V28" s="17" t="n">
-        <v>-2485</v>
+        <v>-1904</v>
       </c>
       <c r="W28" s="18" t="n">
-        <v>-14.7</v>
+        <v>-16.7</v>
       </c>
       <c r="X28" s="2" t="n">
         <v>2</v>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="P29" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23650 PE</t>
+          <t>NIFTY 23550 PE</t>
         </is>
       </c>
       <c r="Q29" s="9" t="inlineStr">
@@ -3522,28 +3522,28 @@
         </is>
       </c>
       <c r="R29" s="11" t="n">
-        <v>138.47</v>
+        <v>95.56999999999999</v>
       </c>
       <c r="S29" s="11" t="n">
-        <v>147.31</v>
+        <v>102.14</v>
       </c>
       <c r="T29" s="13" t="n">
-        <v>9001</v>
+        <v>24848</v>
       </c>
       <c r="U29" s="13" t="n">
-        <v>9575</v>
+        <v>26556</v>
       </c>
       <c r="V29" s="14" t="n">
-        <v>510</v>
+        <v>1612</v>
       </c>
       <c r="W29" s="15" t="n">
-        <v>5.7</v>
+        <v>6.5</v>
       </c>
       <c r="X29" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y29" s="9" t="n">
-        <v>65</v>
+        <v>260</v>
       </c>
       <c r="Z29" s="10" t="inlineStr">
         <is>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23800 PE</t>
+          <t>NIFTY 23700 PE</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
@@ -3624,28 +3624,28 @@
         </is>
       </c>
       <c r="R30" s="4" t="n">
-        <v>60.25</v>
+        <v>22.37</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>83.19</v>
+        <v>33.47</v>
       </c>
       <c r="T30" s="6" t="n">
-        <v>7832</v>
+        <v>5816</v>
       </c>
       <c r="U30" s="6" t="n">
-        <v>10815</v>
+        <v>8702</v>
       </c>
       <c r="V30" s="7" t="n">
-        <v>2916</v>
+        <v>2824</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>37.2</v>
+        <v>48.6</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z30" s="3" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="P31" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23950 CE</t>
+          <t>NIFTY 24050 CE</t>
         </is>
       </c>
       <c r="Q31" s="9" t="inlineStr">
@@ -3726,22 +3726,22 @@
         </is>
       </c>
       <c r="R31" s="11" t="n">
-        <v>123.41</v>
+        <v>78.55</v>
       </c>
       <c r="S31" s="11" t="n">
-        <v>122.49</v>
+        <v>77.67</v>
       </c>
       <c r="T31" s="13" t="n">
-        <v>16043</v>
+        <v>10212</v>
       </c>
       <c r="U31" s="13" t="n">
-        <v>15924</v>
+        <v>10097</v>
       </c>
       <c r="V31" s="20" t="n">
-        <v>-196</v>
+        <v>-180</v>
       </c>
       <c r="W31" s="21" t="n">
-        <v>-1.2</v>
+        <v>-1.8</v>
       </c>
       <c r="X31" s="9" t="n">
         <v>2</v>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23950 PE</t>
+          <t>NIFTY 23850 PE</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
@@ -3828,28 +3828,28 @@
         </is>
       </c>
       <c r="R32" s="4" t="n">
-        <v>142.38</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>163</v>
+        <v>111.26</v>
       </c>
       <c r="T32" s="6" t="n">
-        <v>9255</v>
+        <v>12434</v>
       </c>
       <c r="U32" s="6" t="n">
-        <v>10595</v>
+        <v>14464</v>
       </c>
       <c r="V32" s="7" t="n">
-        <v>1274</v>
+        <v>1956</v>
       </c>
       <c r="W32" s="8" t="n">
-        <v>13.8</v>
+        <v>15.7</v>
       </c>
       <c r="X32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y32" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z32" s="3" t="inlineStr">
         <is>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="P33" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24000 PE</t>
+          <t>NIFTY 23950 PE</t>
         </is>
       </c>
       <c r="Q33" s="9" t="inlineStr">
@@ -3930,28 +3930,28 @@
         </is>
       </c>
       <c r="R33" s="11" t="n">
-        <v>159.9</v>
+        <v>134.93</v>
       </c>
       <c r="S33" s="11" t="n">
-        <v>164.09</v>
+        <v>138.65</v>
       </c>
       <c r="T33" s="13" t="n">
-        <v>20787</v>
+        <v>26311</v>
       </c>
       <c r="U33" s="13" t="n">
-        <v>21332</v>
+        <v>27037</v>
       </c>
       <c r="V33" s="14" t="n">
-        <v>458</v>
+        <v>628</v>
       </c>
       <c r="W33" s="15" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="X33" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y33" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z33" s="10" t="inlineStr">
         <is>
@@ -3977,7 +3977,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24100 CE</t>
+          <t>NIFTY 24200 CE</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
@@ -4032,28 +4032,28 @@
         </is>
       </c>
       <c r="R34" s="4" t="n">
-        <v>154.44</v>
+        <v>109.25</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>134.15</v>
+        <v>93.11</v>
       </c>
       <c r="T34" s="6" t="n">
-        <v>20077</v>
+        <v>28405</v>
       </c>
       <c r="U34" s="6" t="n">
-        <v>17440</v>
+        <v>24209</v>
       </c>
       <c r="V34" s="17" t="n">
-        <v>-2718</v>
+        <v>-4290</v>
       </c>
       <c r="W34" s="18" t="n">
-        <v>-13.5</v>
+        <v>-15.1</v>
       </c>
       <c r="X34" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y34" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z34" s="3" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="P35" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24000 PE</t>
+          <t>NIFTY 23900 PE</t>
         </is>
       </c>
       <c r="Q35" s="9" t="inlineStr">
@@ -4134,28 +4134,28 @@
         </is>
       </c>
       <c r="R35" s="11" t="n">
-        <v>50.61</v>
+        <v>17.87</v>
       </c>
       <c r="S35" s="11" t="n">
-        <v>36.47</v>
+        <v>11.25</v>
       </c>
       <c r="T35" s="13" t="n">
-        <v>6579</v>
+        <v>4646</v>
       </c>
       <c r="U35" s="13" t="n">
-        <v>4741</v>
+        <v>2925</v>
       </c>
       <c r="V35" s="20" t="n">
-        <v>-1895</v>
+        <v>-1775</v>
       </c>
       <c r="W35" s="21" t="n">
-        <v>-28.8</v>
+        <v>-38.2</v>
       </c>
       <c r="X35" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y35" s="9" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z35" s="10" t="inlineStr">
         <is>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24050 PE</t>
+          <t>NIFTY 23950 PE</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
@@ -4236,28 +4236,28 @@
         </is>
       </c>
       <c r="R36" s="4" t="n">
-        <v>63.5</v>
+        <v>24.47</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>61.03</v>
+        <v>22.45</v>
       </c>
       <c r="T36" s="6" t="n">
-        <v>4128</v>
+        <v>4772</v>
       </c>
       <c r="U36" s="6" t="n">
-        <v>3967</v>
+        <v>4378</v>
       </c>
       <c r="V36" s="17" t="n">
-        <v>-215</v>
+        <v>-449</v>
       </c>
       <c r="W36" s="18" t="n">
-        <v>-5.2</v>
+        <v>-9.4</v>
       </c>
       <c r="X36" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y36" s="2" t="n">
-        <v>65</v>
+        <v>195</v>
       </c>
       <c r="Z36" s="3" t="inlineStr">
         <is>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="P37" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24100 PE</t>
+          <t>NIFTY 24050 PE</t>
         </is>
       </c>
       <c r="Q37" s="9" t="inlineStr">
@@ -4338,22 +4338,22 @@
         </is>
       </c>
       <c r="R37" s="11" t="n">
-        <v>122.02</v>
+        <v>97.47</v>
       </c>
       <c r="S37" s="11" t="n">
-        <v>105.43</v>
+        <v>83.11</v>
       </c>
       <c r="T37" s="13" t="n">
-        <v>15863</v>
+        <v>12671</v>
       </c>
       <c r="U37" s="13" t="n">
-        <v>13706</v>
+        <v>10804</v>
       </c>
       <c r="V37" s="20" t="n">
-        <v>-2230</v>
+        <v>-1935</v>
       </c>
       <c r="W37" s="21" t="n">
-        <v>-14.1</v>
+        <v>-15.3</v>
       </c>
       <c r="X37" s="9" t="n">
         <v>2</v>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="P38" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24150 PE</t>
+          <t>NIFTY 24050 PE</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
@@ -4440,28 +4440,28 @@
         </is>
       </c>
       <c r="R38" s="4" t="n">
-        <v>112.26</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>111.33</v>
+        <v>70.09</v>
       </c>
       <c r="T38" s="6" t="n">
-        <v>14594</v>
+        <v>13837</v>
       </c>
       <c r="U38" s="6" t="n">
-        <v>14473</v>
+        <v>13668</v>
       </c>
       <c r="V38" s="17" t="n">
-        <v>-195</v>
+        <v>-242</v>
       </c>
       <c r="W38" s="18" t="n">
-        <v>-1.3</v>
+        <v>-1.7</v>
       </c>
       <c r="X38" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y38" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z38" s="3" t="inlineStr">
         <is>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="P39" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24200 PE</t>
+          <t>NIFTY 24100 PE</t>
         </is>
       </c>
       <c r="Q39" s="9" t="inlineStr">
@@ -4542,22 +4542,22 @@
         </is>
       </c>
       <c r="R39" s="11" t="n">
-        <v>123.77</v>
+        <v>79.56999999999999</v>
       </c>
       <c r="S39" s="11" t="n">
-        <v>144.31</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="T39" s="13" t="n">
-        <v>16090</v>
+        <v>10344</v>
       </c>
       <c r="U39" s="13" t="n">
-        <v>18760</v>
+        <v>12337</v>
       </c>
       <c r="V39" s="14" t="n">
-        <v>2589</v>
+        <v>1924</v>
       </c>
       <c r="W39" s="15" t="n">
-        <v>16.1</v>
+        <v>18.6</v>
       </c>
       <c r="X39" s="9" t="n">
         <v>2</v>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -4635,7 +4635,7 @@
       </c>
       <c r="P40" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24300 PE</t>
+          <t>NIFTY 24200 PE</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
@@ -4644,22 +4644,22 @@
         </is>
       </c>
       <c r="R40" s="4" t="n">
-        <v>138.12</v>
+        <v>93.84999999999999</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>150.48</v>
+        <v>103.12</v>
       </c>
       <c r="T40" s="6" t="n">
-        <v>17956</v>
+        <v>12200</v>
       </c>
       <c r="U40" s="6" t="n">
-        <v>19562</v>
+        <v>13406</v>
       </c>
       <c r="V40" s="7" t="n">
-        <v>1524</v>
+        <v>1134</v>
       </c>
       <c r="W40" s="8" t="n">
-        <v>8.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="X40" s="2" t="n">
         <v>2</v>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>PDH Support Flip</t>
+          <t>PDH Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="P41" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24350 CE</t>
+          <t>NIFTY 24450 CE</t>
         </is>
       </c>
       <c r="Q41" s="9" t="inlineStr">
@@ -4746,22 +4746,22 @@
         </is>
       </c>
       <c r="R41" s="11" t="n">
-        <v>151.85</v>
+        <v>105.33</v>
       </c>
       <c r="S41" s="11" t="n">
-        <v>133.61</v>
+        <v>91.06</v>
       </c>
       <c r="T41" s="13" t="n">
-        <v>19740</v>
+        <v>13693</v>
       </c>
       <c r="U41" s="13" t="n">
-        <v>17369</v>
+        <v>11838</v>
       </c>
       <c r="V41" s="20" t="n">
-        <v>-2452</v>
+        <v>-1925</v>
       </c>
       <c r="W41" s="21" t="n">
-        <v>-12.4</v>
+        <v>-14.1</v>
       </c>
       <c r="X41" s="9" t="n">
         <v>2</v>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="P42" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24150 PE</t>
+          <t>NIFTY 24050 PE</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
@@ -4848,28 +4848,28 @@
         </is>
       </c>
       <c r="R42" s="4" t="n">
-        <v>162.35</v>
+        <v>115.9</v>
       </c>
       <c r="S42" s="4" t="n">
-        <v>145.17</v>
+        <v>102.09</v>
       </c>
       <c r="T42" s="6" t="n">
-        <v>21106</v>
+        <v>30134</v>
       </c>
       <c r="U42" s="6" t="n">
-        <v>18872</v>
+        <v>26543</v>
       </c>
       <c r="V42" s="17" t="n">
-        <v>-2317</v>
+        <v>-3689</v>
       </c>
       <c r="W42" s="18" t="n">
-        <v>-11</v>
+        <v>-12.2</v>
       </c>
       <c r="X42" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y42" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z42" s="3" t="inlineStr">
         <is>
@@ -4895,7 +4895,7 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="P43" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24200 PE</t>
+          <t>NIFTY 24150 PE</t>
         </is>
       </c>
       <c r="Q43" s="9" t="inlineStr">
@@ -4950,22 +4950,22 @@
         </is>
       </c>
       <c r="R43" s="11" t="n">
-        <v>71.92</v>
+        <v>47.42</v>
       </c>
       <c r="S43" s="11" t="n">
-        <v>68.58</v>
+        <v>44.12</v>
       </c>
       <c r="T43" s="13" t="n">
-        <v>9350</v>
+        <v>6165</v>
       </c>
       <c r="U43" s="13" t="n">
-        <v>8915</v>
+        <v>5736</v>
       </c>
       <c r="V43" s="20" t="n">
-        <v>-498</v>
+        <v>-487</v>
       </c>
       <c r="W43" s="21" t="n">
-        <v>-5.3</v>
+        <v>-7.9</v>
       </c>
       <c r="X43" s="9" t="n">
         <v>2</v>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="P44" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24250 PE</t>
+          <t>NIFTY 24150 PE</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr">
@@ -5052,28 +5052,28 @@
         </is>
       </c>
       <c r="R44" s="4" t="n">
-        <v>65.41</v>
+        <v>26.03</v>
       </c>
       <c r="S44" s="4" t="n">
-        <v>105.01</v>
+        <v>47.95</v>
       </c>
       <c r="T44" s="6" t="n">
-        <v>4252</v>
+        <v>5076</v>
       </c>
       <c r="U44" s="6" t="n">
-        <v>6826</v>
+        <v>9350</v>
       </c>
       <c r="V44" s="7" t="n">
-        <v>2515</v>
+        <v>4212</v>
       </c>
       <c r="W44" s="8" t="n">
-        <v>59.1</v>
+        <v>83</v>
       </c>
       <c r="X44" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y44" s="2" t="n">
-        <v>65</v>
+        <v>195</v>
       </c>
       <c r="Z44" s="3" t="inlineStr">
         <is>
@@ -5099,7 +5099,7 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="P45" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24050 PE</t>
+          <t>NIFTY 23950 PE</t>
         </is>
       </c>
       <c r="Q45" s="9" t="inlineStr">
@@ -5154,22 +5154,22 @@
         </is>
       </c>
       <c r="R45" s="11" t="n">
-        <v>146.62</v>
+        <v>100.92</v>
       </c>
       <c r="S45" s="11" t="n">
-        <v>129.18</v>
+        <v>87.36</v>
       </c>
       <c r="T45" s="13" t="n">
-        <v>19061</v>
+        <v>13120</v>
       </c>
       <c r="U45" s="13" t="n">
-        <v>16793</v>
+        <v>11357</v>
       </c>
       <c r="V45" s="20" t="n">
-        <v>-2347</v>
+        <v>-1832</v>
       </c>
       <c r="W45" s="21" t="n">
-        <v>-12.3</v>
+        <v>-14</v>
       </c>
       <c r="X45" s="9" t="n">
         <v>2</v>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="P46" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24200 PE</t>
+          <t>NIFTY 24100 PE</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
@@ -5256,28 +5256,28 @@
         </is>
       </c>
       <c r="R46" s="4" t="n">
-        <v>151.22</v>
+        <v>106.55</v>
       </c>
       <c r="S46" s="4" t="n">
-        <v>152.97</v>
+        <v>107.61</v>
       </c>
       <c r="T46" s="6" t="n">
-        <v>19659</v>
+        <v>27703</v>
       </c>
       <c r="U46" s="6" t="n">
-        <v>19886</v>
+        <v>27979</v>
       </c>
       <c r="V46" s="7" t="n">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="W46" s="8" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="X46" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y46" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z46" s="3" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="P47" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24250 PE</t>
+          <t>NIFTY 24150 PE</t>
         </is>
       </c>
       <c r="Q47" s="9" t="inlineStr">
@@ -5358,28 +5358,28 @@
         </is>
       </c>
       <c r="R47" s="11" t="n">
-        <v>61.66</v>
+        <v>24.43</v>
       </c>
       <c r="S47" s="11" t="n">
-        <v>43.31</v>
+        <v>14.9</v>
       </c>
       <c r="T47" s="13" t="n">
-        <v>8016</v>
+        <v>6352</v>
       </c>
       <c r="U47" s="13" t="n">
-        <v>5630</v>
+        <v>3874</v>
       </c>
       <c r="V47" s="20" t="n">
-        <v>-2444</v>
+        <v>-2533</v>
       </c>
       <c r="W47" s="21" t="n">
-        <v>-30.5</v>
+        <v>-39.9</v>
       </c>
       <c r="X47" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y47" s="9" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z47" s="10" t="inlineStr">
         <is>
@@ -5405,7 +5405,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="P48" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24300 PE</t>
+          <t>NIFTY 24200 PE</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
@@ -5460,28 +5460,28 @@
         </is>
       </c>
       <c r="R48" s="4" t="n">
-        <v>72.01000000000001</v>
+        <v>30.17</v>
       </c>
       <c r="S48" s="4" t="n">
-        <v>95.72</v>
+        <v>43.62</v>
       </c>
       <c r="T48" s="6" t="n">
-        <v>9361</v>
+        <v>5883</v>
       </c>
       <c r="U48" s="6" t="n">
-        <v>12444</v>
+        <v>8506</v>
       </c>
       <c r="V48" s="7" t="n">
-        <v>3013</v>
+        <v>2561</v>
       </c>
       <c r="W48" s="8" t="n">
-        <v>32.2</v>
+        <v>43.5</v>
       </c>
       <c r="X48" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y48" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z48" s="3" t="inlineStr">
         <is>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -5670,22 +5670,22 @@
         <v>192.28</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>10555</v>
+        <v>21109</v>
       </c>
       <c r="U50" s="6" t="n">
-        <v>12498</v>
+        <v>24996</v>
       </c>
       <c r="V50" s="7" t="n">
-        <v>1874</v>
+        <v>3795</v>
       </c>
       <c r="W50" s="8" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="X50" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y50" s="2" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z50" s="3" t="inlineStr">
         <is>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="P51" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24450 PE</t>
+          <t>NIFTY 24350 PE</t>
         </is>
       </c>
       <c r="Q51" s="9" t="inlineStr">
@@ -5766,28 +5766,28 @@
         </is>
       </c>
       <c r="R51" s="11" t="n">
-        <v>166.64</v>
+        <v>121.22</v>
       </c>
       <c r="S51" s="11" t="n">
-        <v>163.36</v>
+        <v>118.25</v>
       </c>
       <c r="T51" s="13" t="n">
-        <v>10832</v>
+        <v>31517</v>
       </c>
       <c r="U51" s="13" t="n">
-        <v>10618</v>
+        <v>30745</v>
       </c>
       <c r="V51" s="20" t="n">
-        <v>-280</v>
+        <v>-877</v>
       </c>
       <c r="W51" s="21" t="n">
-        <v>-2.6</v>
+        <v>-2.8</v>
       </c>
       <c r="X51" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y51" s="9" t="n">
-        <v>65</v>
+        <v>260</v>
       </c>
       <c r="Z51" s="10" t="inlineStr">
         <is>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="P52" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24500 PE</t>
+          <t>NIFTY 24400 PE</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr">
@@ -5868,28 +5868,28 @@
         </is>
       </c>
       <c r="R52" s="4" t="n">
-        <v>177.88</v>
+        <v>130.53</v>
       </c>
       <c r="S52" s="4" t="n">
-        <v>196.35</v>
+        <v>145.5</v>
       </c>
       <c r="T52" s="6" t="n">
-        <v>23124</v>
+        <v>33938</v>
       </c>
       <c r="U52" s="6" t="n">
-        <v>25526</v>
+        <v>37830</v>
       </c>
       <c r="V52" s="7" t="n">
-        <v>2308</v>
+        <v>3776</v>
       </c>
       <c r="W52" s="8" t="n">
-        <v>10</v>
+        <v>11.1</v>
       </c>
       <c r="X52" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y52" s="2" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="Z52" s="3" t="inlineStr">
         <is>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -5976,22 +5976,22 @@
         <v>142.15</v>
       </c>
       <c r="T53" s="13" t="n">
-        <v>10720</v>
+        <v>21440</v>
       </c>
       <c r="U53" s="13" t="n">
-        <v>9240</v>
+        <v>18480</v>
       </c>
       <c r="V53" s="20" t="n">
-        <v>-1545</v>
+        <v>-3043</v>
       </c>
       <c r="W53" s="21" t="n">
-        <v>-14.4</v>
+        <v>-14.2</v>
       </c>
       <c r="X53" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y53" s="9" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="Z53" s="10" t="inlineStr">
         <is>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip</t>
+          <t>PDL Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="P54" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24500 PE</t>
+          <t>NIFTY 24450 PE</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr">
@@ -6072,28 +6072,28 @@
         </is>
       </c>
       <c r="R54" s="4" t="n">
-        <v>166.12</v>
+        <v>141.85</v>
       </c>
       <c r="S54" s="4" t="n">
-        <v>181.47</v>
+        <v>155.69</v>
       </c>
       <c r="T54" s="6" t="n">
-        <v>21596</v>
+        <v>27661</v>
       </c>
       <c r="U54" s="6" t="n">
-        <v>23591</v>
+        <v>30360</v>
       </c>
       <c r="V54" s="7" t="n">
-        <v>1905</v>
+        <v>2596</v>
       </c>
       <c r="W54" s="8" t="n">
-        <v>8.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="X54" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y54" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z54" s="3" t="inlineStr">
         <is>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip</t>
+          <t>OR-30L Resistance Flip [Tier 1 (General]</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="P55" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24550 PE</t>
+          <t>NIFTY 24500 PE</t>
         </is>
       </c>
       <c r="Q55" s="9" t="inlineStr">
@@ -6174,28 +6174,28 @@
         </is>
       </c>
       <c r="R55" s="11" t="n">
-        <v>154.52</v>
+        <v>131.48</v>
       </c>
       <c r="S55" s="11" t="n">
-        <v>178.8</v>
+        <v>153.37</v>
       </c>
       <c r="T55" s="13" t="n">
-        <v>20088</v>
+        <v>25639</v>
       </c>
       <c r="U55" s="13" t="n">
-        <v>23244</v>
+        <v>29907</v>
       </c>
       <c r="V55" s="14" t="n">
-        <v>3067</v>
+        <v>4168</v>
       </c>
       <c r="W55" s="15" t="n">
-        <v>15.3</v>
+        <v>16.3</v>
       </c>
       <c r="X55" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y55" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z55" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(signals): enforce strictly OTM contracts for all telegram alerts and trades
</commit_message>
<xml_diff>
--- a/trades/by_strategy/breakout_and_retest.xlsx
+++ b/trades/by_strategy/breakout_and_retest.xlsx
@@ -713,7 +713,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>OR-30H Support Flip [Tier 3 (Expensive]</t>
+          <t>OR-30H Support Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22700 CE</t>
+          <t>NIFTY 22800 CE</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -768,22 +768,22 @@
         </is>
       </c>
       <c r="R2" s="4" t="n">
-        <v>175.94</v>
+        <v>129.77</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>195.3</v>
+        <v>145.68</v>
       </c>
       <c r="T2" s="6" t="n">
-        <v>22872</v>
+        <v>16870</v>
       </c>
       <c r="U2" s="6" t="n">
-        <v>25389</v>
+        <v>18938</v>
       </c>
       <c r="V2" s="7" t="n">
-        <v>2424</v>
+        <v>1987</v>
       </c>
       <c r="W2" s="8" t="n">
-        <v>10.6</v>
+        <v>11.8</v>
       </c>
       <c r="X2" s="2" t="n">
         <v>2</v>
@@ -815,7 +815,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip [Tier 3 (Expensive]</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22800 PE</t>
+          <t>NIFTY 22700 PE</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
@@ -870,22 +870,22 @@
         </is>
       </c>
       <c r="R3" s="11" t="n">
-        <v>165.38</v>
+        <v>121.21</v>
       </c>
       <c r="S3" s="11" t="n">
-        <v>215.48</v>
+        <v>162.55</v>
       </c>
       <c r="T3" s="13" t="n">
-        <v>21499</v>
+        <v>15757</v>
       </c>
       <c r="U3" s="13" t="n">
-        <v>28012</v>
+        <v>21132</v>
       </c>
       <c r="V3" s="14" t="n">
-        <v>6417</v>
+        <v>5290</v>
       </c>
       <c r="W3" s="15" t="n">
-        <v>29.8</v>
+        <v>33.6</v>
       </c>
       <c r="X3" s="9" t="n">
         <v>2</v>
@@ -917,7 +917,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 22950 PE</t>
+          <t>NIFTY 22850 PE</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -972,22 +972,22 @@
         </is>
       </c>
       <c r="R4" s="4" t="n">
-        <v>183.47</v>
+        <v>136.34</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>162.23</v>
+        <v>118.95</v>
       </c>
       <c r="T4" s="6" t="n">
-        <v>23851</v>
+        <v>17724</v>
       </c>
       <c r="U4" s="6" t="n">
-        <v>21090</v>
+        <v>15464</v>
       </c>
       <c r="V4" s="17" t="n">
-        <v>-2849</v>
+        <v>-2338</v>
       </c>
       <c r="W4" s="18" t="n">
-        <v>-11.9</v>
+        <v>-13.2</v>
       </c>
       <c r="X4" s="2" t="n">
         <v>2</v>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 22600 PE</t>
+          <t>NIFTY 22550 PE</t>
         </is>
       </c>
       <c r="Q15" s="9" t="inlineStr">
@@ -2094,22 +2094,22 @@
         </is>
       </c>
       <c r="R15" s="11" t="n">
-        <v>170.5</v>
+        <v>145.36</v>
       </c>
       <c r="S15" s="11" t="n">
-        <v>152.11</v>
+        <v>128.78</v>
       </c>
       <c r="T15" s="13" t="n">
-        <v>22165</v>
+        <v>18897</v>
       </c>
       <c r="U15" s="13" t="n">
-        <v>19774</v>
+        <v>16741</v>
       </c>
       <c r="V15" s="20" t="n">
-        <v>-2476</v>
+        <v>-2235</v>
       </c>
       <c r="W15" s="21" t="n">
-        <v>-11.2</v>
+        <v>-11.8</v>
       </c>
       <c r="X15" s="9" t="n">
         <v>2</v>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="P49" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24400 PE</t>
+          <t>NIFTY 24300 PE</t>
         </is>
       </c>
       <c r="Q49" s="9" t="inlineStr">
@@ -5562,22 +5562,22 @@
         </is>
       </c>
       <c r="R49" s="11" t="n">
-        <v>162.85</v>
+        <v>115.25</v>
       </c>
       <c r="S49" s="11" t="n">
-        <v>214.25</v>
+        <v>157.06</v>
       </c>
       <c r="T49" s="13" t="n">
-        <v>21170</v>
+        <v>14982</v>
       </c>
       <c r="U49" s="13" t="n">
-        <v>27852</v>
+        <v>20418</v>
       </c>
       <c r="V49" s="14" t="n">
-        <v>6586</v>
+        <v>5353</v>
       </c>
       <c r="W49" s="15" t="n">
-        <v>31.1</v>
+        <v>35.7</v>
       </c>
       <c r="X49" s="9" t="n">
         <v>2</v>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>PDL Resistance Flip [Tier 3 (Expensive]</t>
+          <t>PDL Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="P50" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24450 PE</t>
+          <t>NIFTY 24350 PE</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
@@ -5664,22 +5664,22 @@
         </is>
       </c>
       <c r="R50" s="4" t="n">
-        <v>162.38</v>
+        <v>115.03</v>
       </c>
       <c r="S50" s="4" t="n">
-        <v>192.28</v>
+        <v>139.14</v>
       </c>
       <c r="T50" s="6" t="n">
-        <v>21109</v>
+        <v>14954</v>
       </c>
       <c r="U50" s="6" t="n">
-        <v>24996</v>
+        <v>18088</v>
       </c>
       <c r="V50" s="7" t="n">
-        <v>3795</v>
+        <v>3055</v>
       </c>
       <c r="W50" s="8" t="n">
-        <v>18</v>
+        <v>20.4</v>
       </c>
       <c r="X50" s="2" t="n">
         <v>2</v>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>OR-30L Resistance Flip [Tier 3 (Expensive]</t>
+          <t>OR-30L Resistance Flip [Tier 2 (Super-Trend]</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="P53" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 24600 PE</t>
+          <t>NIFTY 24500 PE</t>
         </is>
       </c>
       <c r="Q53" s="9" t="inlineStr">
@@ -5970,22 +5970,22 @@
         </is>
       </c>
       <c r="R53" s="11" t="n">
-        <v>164.92</v>
+        <v>117.91</v>
       </c>
       <c r="S53" s="11" t="n">
-        <v>142.15</v>
+        <v>99.77</v>
       </c>
       <c r="T53" s="13" t="n">
-        <v>21440</v>
+        <v>15328</v>
       </c>
       <c r="U53" s="13" t="n">
-        <v>18480</v>
+        <v>12970</v>
       </c>
       <c r="V53" s="20" t="n">
-        <v>-3043</v>
+        <v>-2431</v>
       </c>
       <c r="W53" s="21" t="n">
-        <v>-14.2</v>
+        <v>-15.9</v>
       </c>
       <c r="X53" s="9" t="n">
         <v>2</v>

</xml_diff>